<commit_message>
In-progress 2026 data, moving towards initial release
</commit_message>
<xml_diff>
--- a/data/2026/metadata/data_inventory.xlsx
+++ b/data/2026/metadata/data_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/drotto/src/jiflr/data/2026/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E32AD7E5-BB75-244C-81CD-DFC24B303C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524DA853-B3D7-5A45-A75C-FDCA6A3B1EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="2" xr2:uid="{87183E21-210E-514C-A8DD-862AEF854955}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{87183E21-210E-514C-A8DD-862AEF854955}"/>
   </bookViews>
   <sheets>
     <sheet name="on_ice_standard" sheetId="1" r:id="rId1"/>
@@ -181,9 +181,6 @@
     <t>A07</t>
   </si>
   <si>
-    <t>1m sensor placed later than 2m sensor</t>
-  </si>
-  <si>
     <t>F04</t>
   </si>
   <si>
@@ -266,6 +263,9 @@
   </si>
   <si>
     <t>A19</t>
+  </si>
+  <si>
+    <t>1m sensor placed later than 2m sensor. 2m sensor failed to record.</t>
   </si>
 </sst>
 </file>
@@ -687,13 +687,13 @@
         <v>22133624</v>
       </c>
       <c r="F2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -704,7 +704,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D3">
         <v>22133623</v>
@@ -713,13 +713,13 @@
         <v>22133687</v>
       </c>
       <c r="F3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -739,16 +739,16 @@
         <v>22133627</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I4" t="s">
-        <v>46</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -768,13 +768,13 @@
         <v>22133640</v>
       </c>
       <c r="F5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -794,13 +794,13 @@
         <v>22133679</v>
       </c>
       <c r="F6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -820,13 +820,13 @@
         <v>22133630</v>
       </c>
       <c r="F7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -837,7 +837,7 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D8">
         <v>22133635</v>
@@ -846,13 +846,13 @@
         <v>22133680</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -863,7 +863,7 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D9">
         <v>22133663</v>
@@ -872,13 +872,13 @@
         <v>22133650</v>
       </c>
       <c r="F9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -889,7 +889,7 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D10">
         <v>22133672</v>
@@ -898,13 +898,13 @@
         <v>22133652</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -915,7 +915,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D11">
         <v>10383452</v>
@@ -924,13 +924,13 @@
         <v>10568633</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -941,19 +941,19 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D12">
         <v>22133655</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -964,7 +964,7 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D13">
         <v>10383463</v>
@@ -973,13 +973,13 @@
         <v>10383466</v>
       </c>
       <c r="F13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -990,7 +990,7 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D14">
         <v>10568652</v>
@@ -999,13 +999,13 @@
         <v>20102234</v>
       </c>
       <c r="F14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1016,7 +1016,7 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D15">
         <v>10383459</v>
@@ -1025,13 +1025,13 @@
         <v>10568650</v>
       </c>
       <c r="F15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -1042,7 +1042,7 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D16">
         <v>10568610</v>
@@ -1051,13 +1051,13 @@
         <v>10727341</v>
       </c>
       <c r="F16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -1068,7 +1068,7 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D17">
         <v>10383222</v>
@@ -1077,13 +1077,13 @@
         <v>10383221</v>
       </c>
       <c r="F17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -1094,19 +1094,19 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D18">
         <v>22133660</v>
       </c>
       <c r="F18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I18" t="s">
         <v>20</v>
@@ -1120,19 +1120,19 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D19">
         <v>22133639</v>
       </c>
       <c r="F19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I19" t="s">
         <v>20</v>
@@ -1155,13 +1155,13 @@
         <v>22133685</v>
       </c>
       <c r="F20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
@@ -1181,13 +1181,13 @@
         <v>22133686</v>
       </c>
       <c r="F21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -1207,13 +1207,13 @@
         <v>22133676</v>
       </c>
       <c r="F22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -1233,13 +1233,13 @@
         <v>22133674</v>
       </c>
       <c r="F23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -1259,13 +1259,13 @@
         <v>22133675</v>
       </c>
       <c r="F24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
@@ -1285,13 +1285,13 @@
         <v>22133629</v>
       </c>
       <c r="F25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
@@ -1311,13 +1311,13 @@
         <v>22133678</v>
       </c>
       <c r="F26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
@@ -1334,13 +1334,13 @@
         <v>22133653</v>
       </c>
       <c r="F27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I27" t="s">
         <v>20</v>
@@ -1360,13 +1360,13 @@
         <v>22133644</v>
       </c>
       <c r="F28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I28" t="s">
         <v>20</v>
@@ -1386,13 +1386,13 @@
         <v>22133681</v>
       </c>
       <c r="F29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I29" t="s">
         <v>20</v>
@@ -1412,13 +1412,13 @@
         <v>22133664</v>
       </c>
       <c r="F30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I30" t="s">
         <v>20</v>
@@ -1438,13 +1438,13 @@
         <v>22133684</v>
       </c>
       <c r="F31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I31" t="s">
         <v>20</v>
@@ -1464,13 +1464,13 @@
         <v>22133642</v>
       </c>
       <c r="F32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I32" t="s">
         <v>20</v>
@@ -1484,7 +1484,7 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D33">
         <v>22133656</v>
@@ -1493,13 +1493,13 @@
         <v>22133648</v>
       </c>
       <c r="F33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -1510,7 +1510,7 @@
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D34">
         <v>22133662</v>
@@ -1519,13 +1519,13 @@
         <v>22133683</v>
       </c>
       <c r="F34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1594,13 +1594,13 @@
         <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -1623,13 +1623,13 @@
         <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -1652,13 +1652,13 @@
         <v>38</v>
       </c>
       <c r="G4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -1669,7 +1669,7 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D5">
         <v>10568620</v>
@@ -1678,16 +1678,16 @@
         <v>22133634</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -1698,7 +1698,7 @@
         <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D6">
         <v>22038781</v>
@@ -1707,16 +1707,16 @@
         <v>22133646</v>
       </c>
       <c r="F6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1790,19 +1790,19 @@
         <v>11710</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -1828,16 +1828,16 @@
         <v>43</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -1863,13 +1863,13 @@
         <v>44</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -1880,7 +1880,7 @@
         <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D5">
         <v>22133641</v>
@@ -1892,16 +1892,16 @@
         <v>11707</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
@@ -1912,7 +1912,7 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D6">
         <v>22133669</v>
@@ -1924,13 +1924,13 @@
         <v>11709</v>
       </c>
       <c r="H6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -1947,19 +1947,19 @@
         <v>11706</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>